<commit_message>
docs(comms): add Localhost 5-item set tab - route/eat-rest-relax/dice/npc-folders/npcs-met
Uses the smoke-test-workbook skill's builder. All five held unpushed
pending Xero's localhost test; approvable individually per HP.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks/The Tapestry Smoke Testing.xlsx
+++ b/tasks/The Tapestry Smoke Testing.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Mechanics Verify 2026-07-06" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Portrait Bank 2026-08-03" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Onboarding Tour 2026-08-04" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Localhost 5-item set 2026-09-16" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Smoke 2026-07-13'!$A$1:$E$58</definedName>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -100,8 +101,22 @@
       <color rgb="00CCE0F5"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -188,8 +203,23 @@
         <fgColor rgb="002F6FA8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF3EA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -212,11 +242,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -312,6 +356,36 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3592,4 +3666,521 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:F37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" style="31" min="1" max="1"/>
+    <col width="5" customWidth="1" style="31" min="2" max="2"/>
+    <col width="12" customWidth="1" style="31" min="3" max="3"/>
+    <col width="50" customWidth="1" style="31" min="4" max="4"/>
+    <col width="50" customWidth="1" style="31" min="5" max="5"/>
+    <col width="24" customWidth="1" style="31" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="31">
+      <c r="B1" s="44" t="inlineStr">
+        <is>
+          <t>LOCALHOST ONLY - FIVE FEATURES AWAITING YOUR TEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="46.5" customHeight="1" s="31">
+      <c r="B2" s="45" t="inlineStr">
+        <is>
+          <t>All five of these are held UNPUSHED on your local dev server (localhost:3000), not the live site, per the local-first policy. Each is on its own branch, so you can approve them individually - "ship 1 and 3, hold the rest" is a fine answer. Verified before this was written: dev server confirmed up and serving; each feature's code confirmed present in the branch it ships from.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="31">
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>BEFORE YOU START</t>
+        </is>
+      </c>
+      <c r="C4" s="47" t="n"/>
+      <c r="D4" s="47" t="n"/>
+      <c r="E4" s="47" t="n"/>
+      <c r="F4" s="47" t="n"/>
+    </row>
+    <row r="5" ht="17" customHeight="1" s="31">
+      <c r="B5" s="45" t="inlineStr">
+        <is>
+          <t>Make sure your local dev server is running (Start-Tapestry.bat) before starting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1" s="31">
+      <c r="B6" s="45" t="inlineStr">
+        <is>
+          <t>Items 1-3 and 5 (Route tool, Eat/Rest/Relax, Dice roller, NPCs Met) can be tested as the GM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1" s="31">
+      <c r="B7" s="45" t="inlineStr">
+        <is>
+          <t>Item 4 (NPC folders) MUST be tested as a PLAYER - use a second browser or a playtester login, not your GM account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="31" customHeight="1" s="31">
+      <c r="B8" s="45" t="inlineStr">
+        <is>
+          <t>Item 5 (NPCs Met) needs a campaign where the party has actually met at least one NPC (a First Impression rolled) to show anything other than the empty state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="31" customHeight="1" s="31">
+      <c r="B9" s="48" t="inlineStr">
+        <is>
+          <t>NOT on localhost, and you should not go looking for it: the fog-of-war / shared-scene fix. It needs one new database column added first, and localhost and live share the same database - adding it now would break the table page for everyone. It ships once you okay that column.</t>
+        </is>
+      </c>
+      <c r="C9" s="49" t="n"/>
+      <c r="D9" s="49" t="n"/>
+      <c r="E9" s="49" t="n"/>
+      <c r="F9" s="49" t="n"/>
+    </row>
+    <row r="11" ht="62" customHeight="1" s="31">
+      <c r="B11" s="50" t="inlineStr">
+        <is>
+          <t>MARKING THE PASS / FAIL COLUMN: Pass = it did what the row said. Fail = it did not, and you saw enough to say so. Skipped = you chose not to run it. Incomplete = you COULD NOT run it, because an earlier step blocked it or you could not find what the step names. A step blocked by an earlier failure is Incomplete, not Skipped. Incomplete is not a failure: nothing was proven either way, and it tells Comms to fix the step rather than chase a bug.</t>
+        </is>
+      </c>
+      <c r="C11" s="51" t="n"/>
+      <c r="D11" s="51" t="n"/>
+      <c r="E11" s="51" t="n"/>
+      <c r="F11" s="51" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1" s="31">
+      <c r="B13" s="52" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C13" s="52" t="inlineStr">
+        <is>
+          <t>Pass / Fail</t>
+        </is>
+      </c>
+      <c r="D13" s="52" t="inlineStr">
+        <is>
+          <t>What you do</t>
+        </is>
+      </c>
+      <c r="E13" s="52" t="inlineStr">
+        <is>
+          <t>What you should see if it is right</t>
+        </is>
+      </c>
+      <c r="F13" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="31" customHeight="1" s="31">
+      <c r="B14" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="54" t="inlineStr"/>
+      <c r="D14" s="55" t="inlineStr">
+        <is>
+          <t>[ROUTE TOOL] Open a Story you are the GM of, and go to the campaign map.</t>
+        </is>
+      </c>
+      <c r="E14" s="55" t="inlineStr">
+        <is>
+          <t>The map loads normally, as it always has.</t>
+        </is>
+      </c>
+      <c r="F14" s="55" t="inlineStr"/>
+    </row>
+    <row r="15" ht="31" customHeight="1" s="31">
+      <c r="B15" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="54" t="inlineStr"/>
+      <c r="D15" s="55" t="inlineStr">
+        <is>
+          <t>[ROUTE TOOL] Click the ROUTE button, then click two spots on the map to plan a route between them.</t>
+        </is>
+      </c>
+      <c r="E15" s="55" t="inlineStr">
+        <is>
+          <t>A route line is drawn along the roads between the two points you clicked.</t>
+        </is>
+      </c>
+      <c r="F15" s="55" t="inlineStr"/>
+    </row>
+    <row r="16" ht="46.5" customHeight="1" s="31">
+      <c r="B16" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="54" t="inlineStr"/>
+      <c r="D16" s="55" t="inlineStr">
+        <is>
+          <t>[ROUTE TOOL] Find the speed slider and drag it slowly from one end to the other. Read out every label you pass, in order.</t>
+        </is>
+      </c>
+      <c r="E16" s="55" t="inlineStr">
+        <is>
+          <t>The label changes as you drag. Write down the exact labels and order you saw (expected set: Walking, Bike, Horse, Car 22, Car 40, Car 70).</t>
+        </is>
+      </c>
+      <c r="F16" s="55" t="inlineStr"/>
+    </row>
+    <row r="17" ht="31" customHeight="1" s="31">
+      <c r="B17" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="54" t="inlineStr"/>
+      <c r="D17" s="55" t="inlineStr">
+        <is>
+          <t>[ROUTE TOOL] Click the TRAVEL button.</t>
+        </is>
+      </c>
+      <c r="E17" s="55" t="inlineStr">
+        <is>
+          <t>A yellow dot appears on the route line and moves from the start point toward the destination.</t>
+        </is>
+      </c>
+      <c r="F17" s="55" t="inlineStr"/>
+    </row>
+    <row r="18" ht="62" customHeight="1" s="31">
+      <c r="B18" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" s="54" t="inlineStr"/>
+      <c r="D18" s="55" t="inlineStr">
+        <is>
+          <t>[ROUTE TOOL] Watch what the dot does once it reaches the destination, and drag the speed slider while it is still moving.</t>
+        </is>
+      </c>
+      <c r="E18" s="55" t="inlineStr">
+        <is>
+          <t>Report what the dot does at the end (stop, loop back to the start, disappear - whichever it is) and whether dragging the slider mid-travel changes how fast the dot moves.</t>
+        </is>
+      </c>
+      <c r="F18" s="55" t="inlineStr"/>
+    </row>
+    <row r="19" ht="31" customHeight="1" s="31">
+      <c r="B19" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="54" t="inlineStr"/>
+      <c r="D19" s="55" t="inlineStr">
+        <is>
+          <t>[EAT / REST / RELAX] Open the Campaign Sheet, then click the Eat button.</t>
+        </is>
+      </c>
+      <c r="E19" s="55" t="inlineStr">
+        <is>
+          <t>Something happens on screen (not the old placeholder alert) - report exactly what.</t>
+        </is>
+      </c>
+      <c r="F19" s="55" t="inlineStr"/>
+    </row>
+    <row r="20" ht="62" customHeight="1" s="31">
+      <c r="B20" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" s="54" t="inlineStr"/>
+      <c r="D20" s="55" t="inlineStr">
+        <is>
+          <t>[EAT / REST / RELAX] Click the Rest button.</t>
+        </is>
+      </c>
+      <c r="E20" s="55" t="inlineStr">
+        <is>
+          <t>A modal opens with time-length options (Hours / Days / Weeks) and, once you enter at least 8 hours, a Cooling Off checkbox appears. Report what you see and what you are able to set.</t>
+        </is>
+      </c>
+      <c r="F20" s="55" t="inlineStr"/>
+    </row>
+    <row r="21" ht="62" customHeight="1" s="31">
+      <c r="B21" s="53" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" s="54" t="inlineStr"/>
+      <c r="D21" s="55" t="inlineStr">
+        <is>
+          <t>[EAT / REST / RELAX] Close that modal, then click the Relax button.</t>
+        </is>
+      </c>
+      <c r="E21" s="55" t="inlineStr">
+        <is>
+          <t>The same kind of modal opens, but pre-filled to an 8-hour restful rest with Cooling Off already checked (one click should be enough). Report what appears and how it differs from Rest.</t>
+        </is>
+      </c>
+      <c r="F21" s="55" t="inlineStr"/>
+    </row>
+    <row r="22" ht="46.5" customHeight="1" s="31">
+      <c r="B22" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="C22" s="54" t="inlineStr"/>
+      <c r="D22" s="55" t="inlineStr">
+        <is>
+          <t>[DICE ROLLER] Go to the table and find the message box at the bottom of the feed. Click the dice button immediately to the left of it.</t>
+        </is>
+      </c>
+      <c r="E22" s="55" t="inlineStr">
+        <is>
+          <t>A dice panel opens. Report every die button you see in it.</t>
+        </is>
+      </c>
+      <c r="F22" s="55" t="inlineStr"/>
+    </row>
+    <row r="23" ht="31" customHeight="1" s="31">
+      <c r="B23" s="53" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="54" t="inlineStr"/>
+      <c r="D23" s="55" t="inlineStr">
+        <is>
+          <t>[DICE ROLLER] Click the d20 button.</t>
+        </is>
+      </c>
+      <c r="E23" s="55" t="inlineStr">
+        <is>
+          <t>A new line appears in the chat showing a d20 roll. Report the exact line.</t>
+        </is>
+      </c>
+      <c r="F23" s="55" t="inlineStr"/>
+    </row>
+    <row r="24" ht="31" customHeight="1" s="31">
+      <c r="B24" s="53" t="n">
+        <v>11</v>
+      </c>
+      <c r="C24" s="54" t="inlineStr"/>
+      <c r="D24" s="55" t="inlineStr">
+        <is>
+          <t>[DICE ROLLER] Click the + next to where it says "1 die" twice (to get to 3 dice), then click d6.</t>
+        </is>
+      </c>
+      <c r="E24" s="55" t="inlineStr">
+        <is>
+          <t>A new line appears showing 3d6 rolled together. Report the exact line.</t>
+        </is>
+      </c>
+      <c r="F24" s="55" t="inlineStr"/>
+    </row>
+    <row r="25" ht="31" customHeight="1" s="31">
+      <c r="B25" s="53" t="n">
+        <v>12</v>
+      </c>
+      <c r="C25" s="54" t="inlineStr"/>
+      <c r="D25" s="55" t="inlineStr">
+        <is>
+          <t>[DICE ROLLER] Click the + next to the modifier number (starts at 0) three times, then click d20.</t>
+        </is>
+      </c>
+      <c r="E25" s="55" t="inlineStr">
+        <is>
+          <t>A new line appears showing a d20 roll with a +3 modifier applied. Report the exact line.</t>
+        </is>
+      </c>
+      <c r="F25" s="55" t="inlineStr"/>
+    </row>
+    <row r="26" ht="31" customHeight="1" s="31">
+      <c r="B26" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="C26" s="54" t="inlineStr"/>
+      <c r="D26" s="55" t="inlineStr">
+        <is>
+          <t>[DICE ROLLER] Type /r 2d6+3 into the message box and press Enter.</t>
+        </is>
+      </c>
+      <c r="E26" s="55" t="inlineStr">
+        <is>
+          <t>A line appears in the chat showing that roll's result. Report the exact line.</t>
+        </is>
+      </c>
+      <c r="F26" s="55" t="inlineStr"/>
+    </row>
+    <row r="27" ht="77.5" customHeight="1" s="31">
+      <c r="B27" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="C27" s="54" t="inlineStr"/>
+      <c r="D27" s="55" t="inlineStr">
+        <is>
+          <t>[DICE ROLLER] Type /r banana into the message box and press Enter.</t>
+        </is>
+      </c>
+      <c r="E27" s="55" t="inlineStr">
+        <is>
+          <t>This is the important one. It should show an error message INSIDE the dice/chat area and leave what you typed in the box - it should NOT pop up a browser dialog box. Report exactly what you saw, and say plainly whether a popup appeared or not.</t>
+        </is>
+      </c>
+      <c r="F27" s="55" t="inlineStr"/>
+    </row>
+    <row r="28" ht="46.5" customHeight="1" s="31">
+      <c r="B28" s="53" t="n">
+        <v>15</v>
+      </c>
+      <c r="C28" s="54" t="inlineStr"/>
+      <c r="D28" s="55" t="inlineStr">
+        <is>
+          <t>[NPC FOLDERS] Open the Story at localhost as a PLAYER, not the GM (use a second browser or a playtester login). Go to the NPCs tab.</t>
+        </is>
+      </c>
+      <c r="E28" s="55" t="inlineStr">
+        <is>
+          <t>The NPC list loads with its folders, same as the GM sees, but you are logged in as a player.</t>
+        </is>
+      </c>
+      <c r="F28" s="55" t="inlineStr"/>
+    </row>
+    <row r="29" ht="46.5" customHeight="1" s="31">
+      <c r="B29" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="C29" s="54" t="inlineStr"/>
+      <c r="D29" s="55" t="inlineStr">
+        <is>
+          <t>[NPC FOLDERS] Drag an NPC onto a different folder heading, then drag an NPC onto another NPC inside the same folder.</t>
+        </is>
+      </c>
+      <c r="E29" s="55" t="inlineStr">
+        <is>
+          <t>The NPC moves into the new folder, and reordering within a folder changes the order shown. Report what happened for both drags.</t>
+        </is>
+      </c>
+      <c r="F29" s="55" t="inlineStr"/>
+    </row>
+    <row r="30" ht="62" customHeight="1" s="31">
+      <c r="B30" s="53" t="n">
+        <v>17</v>
+      </c>
+      <c r="C30" s="54" t="inlineStr"/>
+      <c r="D30" s="55" t="inlineStr">
+        <is>
+          <t>[NPC FOLDERS] Refresh the page.</t>
+        </is>
+      </c>
+      <c r="E30" s="55" t="inlineStr">
+        <is>
+          <t>THIS IS THE REAL TEST. The folder and order changes you just made should still be there after the refresh - not jumped back to alphabetical. Report which one happened.</t>
+        </is>
+      </c>
+      <c r="F30" s="55" t="inlineStr"/>
+    </row>
+    <row r="31" ht="46.5" customHeight="1" s="31">
+      <c r="B31" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="C31" s="54" t="inlineStr"/>
+      <c r="D31" s="55" t="inlineStr">
+        <is>
+          <t>[NPCS MET] Open the Campaign Sheet for a campaign where the party has actually met some NPCs (First Impressions rolled at some point).</t>
+        </is>
+      </c>
+      <c r="E31" s="55" t="inlineStr">
+        <is>
+          <t>The Campaign Sheet loads as usual.</t>
+        </is>
+      </c>
+      <c r="F31" s="55" t="inlineStr"/>
+    </row>
+    <row r="32" ht="108.5" customHeight="1" s="31">
+      <c r="B32" s="53" t="n">
+        <v>19</v>
+      </c>
+      <c r="C32" s="54" t="inlineStr"/>
+      <c r="D32" s="55" t="inlineStr">
+        <is>
+          <t>[NPCS MET] Look at the grid of panels below the row of action buttons.</t>
+        </is>
+      </c>
+      <c r="E32" s="55" t="inlineStr">
+        <is>
+          <t>A panel headed NPCS MET is there. Report what NPCs are listed and the number on the right of each row (e.g. 2/4 = how many of the party met them, out of how many are at the table). If the panel says "Nobody the party has met yet" for a campaign where no First Impression has ever been rolled, that is correct, not a bug.</t>
+        </is>
+      </c>
+      <c r="F32" s="55" t="inlineStr"/>
+    </row>
+    <row r="33" ht="31" customHeight="1" s="31">
+      <c r="B33" s="53" t="n">
+        <v>20</v>
+      </c>
+      <c r="C33" s="54" t="inlineStr"/>
+      <c r="D33" s="55" t="inlineStr">
+        <is>
+          <t>[NPCS MET] Click one of the rows in that panel.</t>
+        </is>
+      </c>
+      <c r="E33" s="55" t="inlineStr">
+        <is>
+          <t>The card for that same NPC opens - report whether it's the one you clicked.</t>
+        </is>
+      </c>
+      <c r="F33" s="55" t="inlineStr"/>
+    </row>
+    <row r="34" ht="77.5" customHeight="1" s="31">
+      <c r="B34" s="53" t="n">
+        <v>21</v>
+      </c>
+      <c r="C34" s="54" t="inlineStr"/>
+      <c r="D34" s="55" t="inlineStr">
+        <is>
+          <t>[NPCS MET] Think about who you'd expect to see listed.</t>
+        </is>
+      </c>
+      <c r="E34" s="55" t="inlineStr">
+        <is>
+          <t>Report whether anyone you expected is missing. Note: "met" means actually introduced (a First Impression rolled) - an NPC you created but never introduced is not expected to show up, that's correct behavior, not a bug.</t>
+        </is>
+      </c>
+      <c r="F34" s="55" t="inlineStr"/>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="31">
+      <c r="B36" s="46" t="inlineStr">
+        <is>
+          <t>IF ANYTHING FAILS</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="n"/>
+      <c r="D36" s="47" t="n"/>
+      <c r="E36" s="47" t="n"/>
+      <c r="F36" s="47" t="n"/>
+    </row>
+    <row r="37" ht="17" customHeight="1" s="31">
+      <c r="B37" s="45" t="inlineStr">
+        <is>
+          <t>Tell Comms which bracketed section AND which step number failed - e.g. "[DICE ROLLER] step 13" - so it routes to the right fix straight away.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B9:F9"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C14:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Skipped,Incomplete"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>